<commit_message>
Actualizacion de rutas en conexion de datos_V1
</commit_message>
<xml_diff>
--- a/Descargas/ContratoCsgUNICON.xlsx
+++ b/Descargas/ContratoCsgUNICON.xlsx
@@ -3126,13 +3126,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{880EC5B6-BC7E-4E10-9C22-3FBFFE10A339}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1082DD02-2DAF-4CDF-9704-386819C2D3F4}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62E5C8ED-7A05-4AE8-87CA-E72C133C9B27}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BD134A06-588E-4260-BD76-13C3BA959754}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D768C192-0B55-4CBA-AD7D-672DDDDF92AA}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{77E5D39D-7AC1-4895-A2EF-999A86D54B35}"/>
 </file>
</xml_diff>